<commit_message>
Release PBIS 0.10 with guided demo, Wave 1 reports and audited local packages
</commit_message>
<xml_diff>
--- a/outputs/entrega-20260929/llave_evaluacion.xlsx
+++ b/outputs/entrega-20260929/llave_evaluacion.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Llave" sheetId="1" r:id="R663648ec3d1a4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Llave" sheetId="1" r:id="R757a7b44d1b54711"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,16 +60,30 @@
     </x:fill>
   </x:fills>
   <x:borders count="3">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">

</xml_diff>